<commit_message>
ran additional exploration including solar capacity in features for electricity use
</commit_message>
<xml_diff>
--- a/data_processed/results_OLS_kWh_electricity_per_capitaincome.xlsx
+++ b/data_processed/results_OLS_kWh_electricity_per_capitaincome.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0.4706" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0.7917" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1137.996350119706</v>
+        <v>925.6453626749358</v>
       </c>
       <c r="D2" t="n">
-        <v>1.387459524296456e-174</v>
+        <v>2.196399168673274e-286</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.043385933543894</v>
+        <v>25.74144605420481</v>
       </c>
       <c r="D3" t="n">
-        <v>2.032681481720436e-16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -487,10 +487,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11.90642261222924</v>
+        <v>-52.52848150370185</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001736745823511756</v>
+        <v>3.719170348529371e-116</v>
       </c>
     </row>
     <row r="5">
@@ -503,10 +503,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-3.191434300688153</v>
+        <v>-8.332299225490367</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03801665745198198</v>
+        <v>4.718794801416767e-20</v>
       </c>
     </row>
     <row r="6">
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-10.41335402453529</v>
+        <v>-8.930220528660348</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0001480784880510462</v>
+        <v>8.512715264577158e-08</v>
       </c>
     </row>
     <row r="7">
@@ -531,14 +531,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>distance_train</t>
+          <t>distance_depstore</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.003634149970839926</v>
+        <v>-0.01832646701533712</v>
       </c>
       <c r="D7" t="n">
-        <v>8.696158347801635e-14</v>
+        <v>1.075496882291935e-29</v>
       </c>
     </row>
     <row r="8">
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.05404143114886092</v>
+        <v>0.04366387425995394</v>
       </c>
       <c r="D8" t="n">
-        <v>6.616073867534964e-11</v>
+        <v>3.526461383495449e-18</v>
       </c>
     </row>
     <row r="9">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-220.10870481993</v>
+        <v>-103.9126337825557</v>
       </c>
       <c r="D9" t="n">
-        <v>7.83756782646878e-192</v>
+        <v>1.34634394662279e-104</v>
       </c>
     </row>
     <row r="10">
@@ -583,10 +583,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.51923076974185</v>
+        <v>9.821653811169405</v>
       </c>
       <c r="D10" t="n">
-        <v>2.559714606877402e-176</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -599,10 +599,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>77.38631691324547</v>
+        <v>22.5957700284397</v>
       </c>
       <c r="D11" t="n">
-        <v>6.684316096636477e-175</v>
+        <v>1.876699460274125e-31</v>
       </c>
     </row>
     <row r="12">
@@ -615,10 +615,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-799.4658885127023</v>
+        <v>304.4506255703678</v>
       </c>
       <c r="D12" t="n">
-        <v>5.651233608898345e-94</v>
+        <v>1.24109095186503e-29</v>
       </c>
     </row>
     <row r="13">
@@ -627,14 +627,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>distance_depstore</t>
+          <t>solarcapacity</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.03746092591210519</v>
+        <v>-261.0375796179617</v>
       </c>
       <c r="D13" t="n">
-        <v>1.081307173781173e-44</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>